<commit_message>
Unificar la columna en una estructura fija de nueve campos
Las cinco dimensiones usan ahora la misma estructura, siempre en el mismo
orden y sin excepciones: META-CAPACIDAD, OBJETIVO, ENFOQUE, METODOLOGÍA,
TÉCNICA, MARCO, ARTEFACTO, CALIDAD Y ÉTICA, COMPETENCIAS.

Antes cada dimensión traía los bloques que le tocaban, lo que hacía que
la comparación entre dimensiones dependiera de cómo estuviera redactada
cada celda. Se eliminan los códigos T0-T9 del texto de la columna: la
etiqueta en palabras basta y se lee sin diccionario al lado.

Dos integraciones para no romper la estructura: las palancas conductuales
de D3 pasan a TÉCNICA, y ResearchOps/BehavioralOps/KnowledgeOps de D5
pasan a METODOLOGÍA.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tAd4V47q1GQgexet1HAzR
</commit_message>
<xml_diff>
--- a/matriz-expertiz/Propuesta_Matriz_expertiz_taxonomias.xlsx
+++ b/matriz-expertiz/Propuesta_Matriz_expertiz_taxonomias.xlsx
@@ -710,10 +710,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="51" customHeight="1">
+    <row r="16" ht="111" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0 Meta-capacidad → T1 Objetivo → T2 Enfoque → T3 Metodología → T4 Técnica → T5 Marco conceptual → T6 Artefacto → T7 Calidad y ética (T7b Ética del liderazgo donde corresponde) → T8 Práctica operativa → T9 Competencia transversal.</t>
+          <t>Las cinco dimensiones usan la MISMA estructura de nueve campos, siempre en este orden y sin excepciones:
+  META-CAPACIDAD → OBJETIVO → ENFOQUE → METODOLOGÍA → TÉCNICA → MARCO → ARTEFACTO → CALIDAD Y ÉTICA → COMPETENCIAS
+Que la estructura sea idéntica es lo que hace comparables las cinco dimensiones entre sí: si un campo estuviera en unas y no en otras, la comparación volvería a depender de cómo esté redactada cada celda.
+Dos integraciones para no romper la estructura: las palancas conductuales de D3 viven dentro de TÉCNICA (son el instrumento de la intervención), y ResearchOps, BehavioralOps y KnowledgeOps de D5 viven dentro de METODOLOGÍA (son la forma de estructurar el trabajo, no un instrumento suelto).</t>
         </is>
       </c>
     </row>
@@ -4763,15 +4766,15 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Estrategia de investigación: componer objetivo, enfoque, metodología y técnicas de forma coherente con la decisión que se necesita tomar. ¿Es esta la investigación que la decisión necesita, o solo la que sabemos hacer?
-T1 OBJETIVO · Problem framing (de decisión de negocio a pregunta de investigación y conducta objetivo); exploración de necesidades, experiencias y contexto; diagnóstico conductual; diagnóstico sistémico.
-T2 ENFOQUE · Cualitativo, cuantitativo y mixto; evidencia primaria y secundaria.
-T3 METODOLOGÍA · Desk research (evidencia secundaria); investigación en campo / etnográfica; estudios longitudinales y de seguimiento.
-T4 TÉCNICA · Recolección: entrevistas, observación estructurada, diarios, encuestas, intercept y mystery shopping (campo físico), analítica de comportamiento. Análisis: diseño muestral, codificación, triangulación de métodos y fuentes, síntesis.
-T5 MARCO · Frameworks de ciencias del comportamiento para leer conducta (COM-B, EAST); systems thinking.
-T6 ARTEFACTO · Insight; plan y estrategia de investigación.
-T7 CALIDAD Y ÉTICA · Calidad y suficiencia de la evidencia; gestión de sesgos; límites de validez; consentimiento y privacidad.
-T9 COMPETENCIA · Pensamiento crítico.</t>
+          <t>META-CAPACIDAD: Estrategia de investigación: componer objetivo, enfoque, metodología y técnicas de forma coherente con la decisión que se necesita tomar.
+OBJETIVO: Problem framing (de decisión de negocio a pregunta de investigación y conducta objetivo); exploración de necesidades, experiencias y contexto; diagnóstico conductual; diagnóstico sistémico.
+ENFOQUE: Cualitativo, cuantitativo y mixto; evidencia primaria y secundaria.
+METODOLOGÍA: Desk research (evidencia secundaria); investigación en campo / etnográfica; estudios longitudinales y de seguimiento.
+TÉCNICA: Recolección: entrevistas, observación estructurada, diarios, encuestas, intercept y mystery shopping (campo físico), analítica de comportamiento. Análisis: diseño muestral, codificación, triangulación de métodos y fuentes, síntesis.
+MARCO: Frameworks de ciencias del comportamiento para leer conducta (COM-B, EAST); systems thinking.
+ARTEFACTO: Insight; plan y estrategia de investigación.
+CALIDAD Y ÉTICA: Calidad y suficiencia de la evidencia; gestión de sesgos; límites de validez; consentimiento y privacidad.
+COMPETENCIAS: Pensamiento crítico.</t>
         </is>
       </c>
     </row>
@@ -4791,13 +4794,15 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Juicio estratégico: decidir qué problema merece resolverse y con cuánta evidencia basta para decidirlo, haciendo explícito el riesgo de equivocarse.
-T1 OBJETIVO · Problem reframing; opportunity framing; formulación y priorización de hipótesis estratégicas.
-T5 MARCO · Frameworks de Research, Design y Behavioral Science (COM-B, EAST, MINDSPACE); systems thinking; teoría del cambio.
-T4 TÉCNICA (análisis y decisión) · Síntesis estratégica; evaluación de valor, viabilidad, riesgo y esfuerzo; matrices de priorización; exploración de escenarios y trade-offs.
-T6 ARTEFACTO · Problema reencuadrado; mapa de oportunidades; hipótesis priorizadas; narrativa estratégica.
-T7 CALIDAD Y ÉTICA · Supuestos explícitos; estándar de evidencia exigible según el tipo de decisión; ética de la intervención.
-T9 COMPETENCIA · Pensamiento crítico; business acumen; storytelling estratégico.</t>
+          <t>META-CAPACIDAD: Juicio estratégico: decidir qué problema merece resolverse y con cuánta evidencia basta para decidirlo, haciendo explícito el riesgo de equivocarse.
+OBJETIVO: Problem reframing; opportunity framing; formulación y priorización de hipótesis estratégicas; definición de direcciones y de trade-offs.
+ENFOQUE: Integración de la evidencia de usuario, de comportamiento y de negocio; lectura divergente para abrir alternativas y convergente para cerrar la decisión; evidencia primaria, secundaria y de mercado.
+METODOLOGÍA: Síntesis estratégica sobre evidencia acumulada; análisis del espacio de problema y de oportunidades; análisis de escenarios; modelado de sistemas y de actores.
+TÉCNICA: Encuadre: árboles de problema, reformulación de la pregunta, mapas de oportunidad. Decisión: matrices de priorización, evaluación de valor, viabilidad, riesgo y esfuerzo, análisis de trade-offs, pre-mortem.
+MARCO: Frameworks de Research, Design y Behavioral Science (COM-B, EAST, MINDSPACE); systems thinking; teoría del cambio; modelos de negocio y de valor.
+ARTEFACTO: Problema reencuadrado; mapa de oportunidades; hipótesis priorizadas; narrativa estratégica de la decisión.
+CALIDAD Y ÉTICA: Supuestos explícitos y trazables; estándar de evidencia exigible según el tipo de decisión; declaración del riesgo de equivocarse; ética de la intervención propuesta.
+COMPETENCIAS: Pensamiento crítico; business acumen; storytelling estratégico.</t>
         </is>
       </c>
     </row>
@@ -4817,15 +4822,15 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>E3 ESPECIALIDAD · Diseño conductual (única especialidad de diseño evaluada por esta matriz).
-T0 META-CAPACIDAD · Criterio de intervención: decidir cuánta intervención pide una conducta, elegir la palanca proporcional al problema y al riesgo ético, y reconocer cuándo lo correcto es no intervenir.
-T1 OBJETIVO · Traducir evidencia y estrategia en principios, conceptos e intervenciones; intervenir sobre una conducta objetivo; orquestar la experiencia a través de touchpoints y canales.
-T5 MARCO · Arquitectura de decisiones; journey thinking; systems thinking.
-T5b PALANCAS DE INTERVENCIÓN · Fricción y esfuerzo; defaults; timing y saliencia; framing y comunicación conductual; incentivos; normas sociales; personalización.
-T4 TÉCNICA · Ideación y conceptualización; traducción de insights a criterios de diseño; prototipado conceptual; behavioral walkthrough; diseño de contenido conductual.
-T6 ARTEFACTO · Principios y criterios de diseño; concepto de intervención; blueprint de orquestación.
-T7 CALIDAD Y ÉTICA · Ética de la influencia (transparencia, autonomía de la persona, no explotación de sesgos); testeabilidad de la intervención.
-X MODELO DE COLABORACIÓN (no es capacidad; describe alcance) · Acompañamiento a Product y Service Design en la conceptualización y orquestación de la experiencia.</t>
+          <t>META-CAPACIDAD: Criterio de intervención: decidir cuánta intervención pide una conducta, elegir la palanca proporcional al problema y al riesgo ético, y reconocer cuándo lo correcto es no intervenir.
+OBJETIVO: Traducir evidencia y estrategia en principios, conceptos e intervenciones; modificar una conducta objetivo; orquestar la experiencia a través de touchpoints y canales.
+ENFOQUE: Diseño conductual, única especialidad de diseño de la matriz. Se diseña sobre conducta observada y no sobre conducta declarada; intervención puntual frente a sistema de intervenciones; reducir fricción frente a añadir refuerzo.
+METODOLOGÍA: Diseño de intervenciones conductuales; arquitectura de decisiones aplicada a un journey; ciclos iterativos de concepto, prueba y ajuste; co-diseño con las áreas dueñas de la experiencia.
+TÉCNICA: Palancas: fricción y esfuerzo, defaults, timing y saliencia, framing y comunicación conductual, incentivos, normas sociales, personalización. Proceso: traducción de insights a criterios de diseño, ideación y conceptualización, prototipado conceptual, behavioral walkthrough, diseño de contenido conductual.
+MARCO: Arquitectura de decisiones; journey thinking; systems thinking; taxonomías de palancas y de sesgos.
+ARTEFACTO: Principios y criterios de diseño; concepto de intervención; prototipo conceptual; blueprint de orquestación; hipótesis conductual lista para validar.
+CALIDAD Y ÉTICA: Ética de la influencia — transparencia, autonomía de la persona, no explotación de sesgos, reversibilidad de la intervención; proporcionalidad entre el problema y la palanca; testeabilidad; equidad del efecto entre segmentos.
+COMPETENCIAS: Pensamiento crítico aplicado al propio diseño; comunicación visual y narrativa del concepto; escucha y traducción entre disciplinas.</t>
         </is>
       </c>
     </row>
@@ -4845,14 +4850,15 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Criterio de evidencia: decidir cuánto rigor exige cada decisión y cuánto sería desperdiciarlo, ajustando el diseño al costo, al riesgo y a la reversibilidad.
-T1 OBJETIVO · UX validation (concepto, prototipo, experiencia); evaluación del efecto de intervenciones conductuales; evaluación de impacto; decisión de iterar, escalar o detener.
-T2 ENFOQUE · Observacional frente a experimental; cuantitativo, cualitativo de validación y mixto.
-T3 METODOLOGÍA · Diseño experimental; RCT; cuasi-experimentos; pre-post con grupo de control; pruebas de concepto y prototipo; piloto en campo (físico) y en producto (digital).
-T4 TÉCNICA · Formulación operacional de hipótesis y variables; A/B testing y multivariante; concept &amp; prototype testing; usability testing; analytics e instrumentación; análisis estadístico.
-T5 MARCO · Inferencia causal; teoría del cambio; jerarquía de evidencia.
-T6 ARTEFACTO · Hipótesis operacionalizada; métricas y criterios de éxito; lectura de resultados y recomendación de decisión.
-T7 CALIDAD Y ÉTICA · Validez interna y externa; control de variables; potencia y tamaño muestral; triangulación como criterio de robustez; ética experimental (consentimiento, grupos de control, reversibilidad).</t>
+          <t>META-CAPACIDAD: Criterio de evidencia: decidir cuánto rigor exige cada decisión y cuánto sería desperdiciarlo, ajustando el diseño al costo, al riesgo y a la reversibilidad.
+OBJETIVO: UX validation (concepto, prototipo, experiencia); evaluación del efecto de las intervenciones conductuales; evaluación de impacto; decisión de iterar, escalar o detener.
+ENFOQUE: Observacional frente a experimental; cuantitativo, cualitativo de validación y mixto; medición en condiciones controladas frente a medición en condiciones reales.
+METODOLOGÍA: Diseño experimental; RCT; cuasi-experimentos por sede, territorio o cohorte; pre-post con grupo de control; pruebas de concepto y de prototipo; piloto en campo (físico) y en producto (digital).
+TÉCNICA: Diseño: operacionalización de hipótesis y variables, definición de grupos y regla de asignación, cálculo de tamaño muestral. Ejecución y análisis: A/B testing y multivariante, concept &amp; prototype testing, usability testing, analytics e instrumentación, análisis estadístico y por segmentos.
+MARCO: Inferencia causal; teoría del cambio; jerarquía de evidencia; modelo lógico de la intervención (el mecanismo por el que se espera que funcione).
+ARTEFACTO: Hipótesis operacionalizada; métricas y criterios de éxito definidos antes de medir; lectura de resultados con tamaño de efecto; recomendación de decisión.
+CALIDAD Y ÉTICA: Validez interna y externa; control de variables; potencia y tamaño muestral; triangulación como criterio de robustez; ética experimental — consentimiento, uso de grupos de control, reversibilidad y no daño al grupo no expuesto.
+COMPETENCIAS: Honestidad intelectual ante resultados negativos; comunicación de la incertidumbre; rigor en la lectura de datos ajenos.</t>
         </is>
       </c>
     </row>
@@ -4872,13 +4878,15 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Criterio de escalamiento y liderazgo: decidir qué se estandariza, qué se deja variar y a qué ritmo se le puede exigir a un equipo, sosteniendo el equilibrio entre lo que el equipo produce y lo que el equipo puede sostener.
-T1 OBJETIVO · Escalar conocimiento, prácticas y capacidades; sostener la decisión basada en evidencia.
-T8 PRÁCTICA OPERATIVA · ResearchOps; BehavioralOps; KnowledgeOps; gestión y activación del conocimiento; repositorios y trazabilidad; automatización; capability building; mejora continua.
-T7 GOBERNANZA, CALIDAD Y ÉTICA · Estándares metodológicos; gobernanza de datos y privacidad; gestión de calidad; ética aplicada.
-T7b ÉTICA DEL LIDERAZGO · Se mide en dos partes que no se mezclan. EQUILIBRIO (se pondera): productividad del equipo ↔ satisfacción del equipo con la persona que lidera, leídas en el mismo periodo y nunca por separado. UMBRAL (se verifica, no se pondera): respeto básico — sin acoso, sin mansplaining, sin conductas excluyentes. El umbral no entra en la ponderación: su incumplimiento verificado bloquea el nivel. Ver hoja «4. Ética del liderazgo».
-T6 ARTEFACTO · Estándares y playbooks; repositorio de evidencia; catálogo de intervenciones reutilizables; modelo de capacidades del Council.
-T9 COMPETENCIA · Stakeholder management; influencia; comunicación estratégica; facilitación; mentoring; priorización de portafolio.</t>
+          <t>META-CAPACIDAD: Criterio de escalamiento y liderazgo: decidir qué se estandariza, qué se deja variar y a qué ritmo se le puede exigir a un equipo, sosteniendo el equilibrio entre lo que el equipo produce y lo que el equipo puede sostener.
+OBJETIVO: Escalar conocimiento, prácticas y capacidades; desarrollar personas; sostener una cultura de decisión basada en evidencia.
+ENFOQUE: Evidencia acumulativa frente a estudio aislado; estandarizar frente a dejar variar; construir capacidad interna frente a resolver por encargo.
+METODOLOGÍA: ResearchOps, BehavioralOps y KnowledgeOps como sistemas de trabajo; gobernanza de estándares y de datos; capability building y modelos de desarrollo de personas; mejora continua.
+TÉCNICA: Conocimiento: repositorios y taxonomías de evidencia, activación y democratización del conocimiento, automatización de tareas operativas, trazabilidad. Liderazgo y equipo: feedback ascendente anónimo, observación estructurada de reuniones (habla, interrupciones y atribución de ideas), registro de asignación de oportunidades visibles, planes de desarrollo, entrevista de salida.
+MARCO: Systems thinking aplicado a la propia capacidad; modelo de madurez de la práctica; ciclo de mejora continua; el propio marco conductual aplicado al equipo — la conducta de quien lidera también es conducta observable.
+ARTEFACTO: Estándares y playbooks; repositorio de evidencia; catálogo de intervenciones reutilizables; modelo de capacidades del Council; tablero del equilibrio productividad–satisfacción del equipo.
+CALIDAD Y ÉTICA: Estándares metodológicos; gobernanza de datos, privacidad y trazabilidad; gestión de calidad. Ética del liderazgo, en dos partes que no se mezclan. EQUILIBRIO (se pondera): productividad del equipo ↔ satisfacción del equipo con la persona que lidera, leídas en el mismo periodo y nunca por separado. UMBRAL (se verifica, no se pondera): respeto básico, sin acoso, sin mansplaining, sin conductas excluyentes; su incumplimiento verificado bloquea el nivel y no entra en la ponderación.
+COMPETENCIAS: Stakeholder management; influencia; comunicación estratégica; facilitación; mentoring; priorización de portafolio.</t>
         </is>
       </c>
     </row>
@@ -5008,15 +5016,15 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Estrategia de investigación: componer objetivo, enfoque, metodología y técnicas de forma coherente con la decisión que se necesita tomar. ¿Es esta la investigación que la decisión necesita, o solo la que sabemos hacer?
-T1 OBJETIVO · Problem framing (de decisión de negocio a pregunta de investigación y conducta objetivo); exploración de necesidades, experiencias y contexto; diagnóstico conductual; diagnóstico sistémico.
-T2 ENFOQUE · Cualitativo, cuantitativo y mixto; evidencia primaria y secundaria.
-T3 METODOLOGÍA · Desk research (evidencia secundaria); investigación en campo / etnográfica; estudios longitudinales y de seguimiento.
-T4 TÉCNICA · Recolección: entrevistas, observación estructurada, diarios, encuestas, intercept y mystery shopping (campo físico), analítica de comportamiento. Análisis: diseño muestral, codificación, triangulación de métodos y fuentes, síntesis.
-T5 MARCO · Frameworks de ciencias del comportamiento para leer conducta (COM-B, EAST); systems thinking.
-T6 ARTEFACTO · Insight; plan y estrategia de investigación.
-T7 CALIDAD Y ÉTICA · Calidad y suficiencia de la evidencia; gestión de sesgos; límites de validez; consentimiento y privacidad.
-T9 COMPETENCIA · Pensamiento crítico.</t>
+          <t>META-CAPACIDAD: Estrategia de investigación: componer objetivo, enfoque, metodología y técnicas de forma coherente con la decisión que se necesita tomar.
+OBJETIVO: Problem framing (de decisión de negocio a pregunta de investigación y conducta objetivo); exploración de necesidades, experiencias y contexto; diagnóstico conductual; diagnóstico sistémico.
+ENFOQUE: Cualitativo, cuantitativo y mixto; evidencia primaria y secundaria.
+METODOLOGÍA: Desk research (evidencia secundaria); investigación en campo / etnográfica; estudios longitudinales y de seguimiento.
+TÉCNICA: Recolección: entrevistas, observación estructurada, diarios, encuestas, intercept y mystery shopping (campo físico), analítica de comportamiento. Análisis: diseño muestral, codificación, triangulación de métodos y fuentes, síntesis.
+MARCO: Frameworks de ciencias del comportamiento para leer conducta (COM-B, EAST); systems thinking.
+ARTEFACTO: Insight; plan y estrategia de investigación.
+CALIDAD Y ÉTICA: Calidad y suficiencia de la evidencia; gestión de sesgos; límites de validez; consentimiento y privacidad.
+COMPETENCIAS: Pensamiento crítico.</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -5076,13 +5084,15 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Juicio estratégico: decidir qué problema merece resolverse y con cuánta evidencia basta para decidirlo, haciendo explícito el riesgo de equivocarse.
-T1 OBJETIVO · Problem reframing; opportunity framing; formulación y priorización de hipótesis estratégicas.
-T5 MARCO · Frameworks de Research, Design y Behavioral Science (COM-B, EAST, MINDSPACE); systems thinking; teoría del cambio.
-T4 TÉCNICA (análisis y decisión) · Síntesis estratégica; evaluación de valor, viabilidad, riesgo y esfuerzo; matrices de priorización; exploración de escenarios y trade-offs.
-T6 ARTEFACTO · Problema reencuadrado; mapa de oportunidades; hipótesis priorizadas; narrativa estratégica.
-T7 CALIDAD Y ÉTICA · Supuestos explícitos; estándar de evidencia exigible según el tipo de decisión; ética de la intervención.
-T9 COMPETENCIA · Pensamiento crítico; business acumen; storytelling estratégico.</t>
+          <t>META-CAPACIDAD: Juicio estratégico: decidir qué problema merece resolverse y con cuánta evidencia basta para decidirlo, haciendo explícito el riesgo de equivocarse.
+OBJETIVO: Problem reframing; opportunity framing; formulación y priorización de hipótesis estratégicas; definición de direcciones y de trade-offs.
+ENFOQUE: Integración de la evidencia de usuario, de comportamiento y de negocio; lectura divergente para abrir alternativas y convergente para cerrar la decisión; evidencia primaria, secundaria y de mercado.
+METODOLOGÍA: Síntesis estratégica sobre evidencia acumulada; análisis del espacio de problema y de oportunidades; análisis de escenarios; modelado de sistemas y de actores.
+TÉCNICA: Encuadre: árboles de problema, reformulación de la pregunta, mapas de oportunidad. Decisión: matrices de priorización, evaluación de valor, viabilidad, riesgo y esfuerzo, análisis de trade-offs, pre-mortem.
+MARCO: Frameworks de Research, Design y Behavioral Science (COM-B, EAST, MINDSPACE); systems thinking; teoría del cambio; modelos de negocio y de valor.
+ARTEFACTO: Problema reencuadrado; mapa de oportunidades; hipótesis priorizadas; narrativa estratégica de la decisión.
+CALIDAD Y ÉTICA: Supuestos explícitos y trazables; estándar de evidencia exigible según el tipo de decisión; declaración del riesgo de equivocarse; ética de la intervención propuesta.
+COMPETENCIAS: Pensamiento crítico; business acumen; storytelling estratégico.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -5142,15 +5152,15 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>E3 ESPECIALIDAD · Diseño conductual (única especialidad de diseño evaluada por esta matriz).
-T0 META-CAPACIDAD · Criterio de intervención: decidir cuánta intervención pide una conducta, elegir la palanca proporcional al problema y al riesgo ético, y reconocer cuándo lo correcto es no intervenir.
-T1 OBJETIVO · Traducir evidencia y estrategia en principios, conceptos e intervenciones; intervenir sobre una conducta objetivo; orquestar la experiencia a través de touchpoints y canales.
-T5 MARCO · Arquitectura de decisiones; journey thinking; systems thinking.
-T5b PALANCAS DE INTERVENCIÓN · Fricción y esfuerzo; defaults; timing y saliencia; framing y comunicación conductual; incentivos; normas sociales; personalización.
-T4 TÉCNICA · Ideación y conceptualización; traducción de insights a criterios de diseño; prototipado conceptual; behavioral walkthrough; diseño de contenido conductual.
-T6 ARTEFACTO · Principios y criterios de diseño; concepto de intervención; blueprint de orquestación.
-T7 CALIDAD Y ÉTICA · Ética de la influencia (transparencia, autonomía de la persona, no explotación de sesgos); testeabilidad de la intervención.
-X MODELO DE COLABORACIÓN (no es capacidad; describe alcance) · Acompañamiento a Product y Service Design en la conceptualización y orquestación de la experiencia.</t>
+          <t>META-CAPACIDAD: Criterio de intervención: decidir cuánta intervención pide una conducta, elegir la palanca proporcional al problema y al riesgo ético, y reconocer cuándo lo correcto es no intervenir.
+OBJETIVO: Traducir evidencia y estrategia en principios, conceptos e intervenciones; modificar una conducta objetivo; orquestar la experiencia a través de touchpoints y canales.
+ENFOQUE: Diseño conductual, única especialidad de diseño de la matriz. Se diseña sobre conducta observada y no sobre conducta declarada; intervención puntual frente a sistema de intervenciones; reducir fricción frente a añadir refuerzo.
+METODOLOGÍA: Diseño de intervenciones conductuales; arquitectura de decisiones aplicada a un journey; ciclos iterativos de concepto, prueba y ajuste; co-diseño con las áreas dueñas de la experiencia.
+TÉCNICA: Palancas: fricción y esfuerzo, defaults, timing y saliencia, framing y comunicación conductual, incentivos, normas sociales, personalización. Proceso: traducción de insights a criterios de diseño, ideación y conceptualización, prototipado conceptual, behavioral walkthrough, diseño de contenido conductual.
+MARCO: Arquitectura de decisiones; journey thinking; systems thinking; taxonomías de palancas y de sesgos.
+ARTEFACTO: Principios y criterios de diseño; concepto de intervención; prototipo conceptual; blueprint de orquestación; hipótesis conductual lista para validar.
+CALIDAD Y ÉTICA: Ética de la influencia — transparencia, autonomía de la persona, no explotación de sesgos, reversibilidad de la intervención; proporcionalidad entre el problema y la palanca; testeabilidad; equidad del efecto entre segmentos.
+COMPETENCIAS: Pensamiento crítico aplicado al propio diseño; comunicación visual y narrativa del concepto; escucha y traducción entre disciplinas.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -5210,14 +5220,15 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Criterio de evidencia: decidir cuánto rigor exige cada decisión y cuánto sería desperdiciarlo, ajustando el diseño al costo, al riesgo y a la reversibilidad.
-T1 OBJETIVO · UX validation (concepto, prototipo, experiencia); evaluación del efecto de intervenciones conductuales; evaluación de impacto; decisión de iterar, escalar o detener.
-T2 ENFOQUE · Observacional frente a experimental; cuantitativo, cualitativo de validación y mixto.
-T3 METODOLOGÍA · Diseño experimental; RCT; cuasi-experimentos; pre-post con grupo de control; pruebas de concepto y prototipo; piloto en campo (físico) y en producto (digital).
-T4 TÉCNICA · Formulación operacional de hipótesis y variables; A/B testing y multivariante; concept &amp; prototype testing; usability testing; analytics e instrumentación; análisis estadístico.
-T5 MARCO · Inferencia causal; teoría del cambio; jerarquía de evidencia.
-T6 ARTEFACTO · Hipótesis operacionalizada; métricas y criterios de éxito; lectura de resultados y recomendación de decisión.
-T7 CALIDAD Y ÉTICA · Validez interna y externa; control de variables; potencia y tamaño muestral; triangulación como criterio de robustez; ética experimental (consentimiento, grupos de control, reversibilidad).</t>
+          <t>META-CAPACIDAD: Criterio de evidencia: decidir cuánto rigor exige cada decisión y cuánto sería desperdiciarlo, ajustando el diseño al costo, al riesgo y a la reversibilidad.
+OBJETIVO: UX validation (concepto, prototipo, experiencia); evaluación del efecto de las intervenciones conductuales; evaluación de impacto; decisión de iterar, escalar o detener.
+ENFOQUE: Observacional frente a experimental; cuantitativo, cualitativo de validación y mixto; medición en condiciones controladas frente a medición en condiciones reales.
+METODOLOGÍA: Diseño experimental; RCT; cuasi-experimentos por sede, territorio o cohorte; pre-post con grupo de control; pruebas de concepto y de prototipo; piloto en campo (físico) y en producto (digital).
+TÉCNICA: Diseño: operacionalización de hipótesis y variables, definición de grupos y regla de asignación, cálculo de tamaño muestral. Ejecución y análisis: A/B testing y multivariante, concept &amp; prototype testing, usability testing, analytics e instrumentación, análisis estadístico y por segmentos.
+MARCO: Inferencia causal; teoría del cambio; jerarquía de evidencia; modelo lógico de la intervención (el mecanismo por el que se espera que funcione).
+ARTEFACTO: Hipótesis operacionalizada; métricas y criterios de éxito definidos antes de medir; lectura de resultados con tamaño de efecto; recomendación de decisión.
+CALIDAD Y ÉTICA: Validez interna y externa; control de variables; potencia y tamaño muestral; triangulación como criterio de robustez; ética experimental — consentimiento, uso de grupos de control, reversibilidad y no daño al grupo no expuesto.
+COMPETENCIAS: Honestidad intelectual ante resultados negativos; comunicación de la incertidumbre; rigor en la lectura de datos ajenos.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -5277,13 +5288,15 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>T0 META-CAPACIDAD · Criterio de escalamiento y liderazgo: decidir qué se estandariza, qué se deja variar y a qué ritmo se le puede exigir a un equipo, sosteniendo el equilibrio entre lo que el equipo produce y lo que el equipo puede sostener.
-T1 OBJETIVO · Escalar conocimiento, prácticas y capacidades; sostener la decisión basada en evidencia.
-T8 PRÁCTICA OPERATIVA · ResearchOps; BehavioralOps; KnowledgeOps; gestión y activación del conocimiento; repositorios y trazabilidad; automatización; capability building; mejora continua.
-T7 GOBERNANZA, CALIDAD Y ÉTICA · Estándares metodológicos; gobernanza de datos y privacidad; gestión de calidad; ética aplicada.
-T7b ÉTICA DEL LIDERAZGO · Se mide en dos partes que no se mezclan. EQUILIBRIO (se pondera): productividad del equipo ↔ satisfacción del equipo con la persona que lidera, leídas en el mismo periodo y nunca por separado. UMBRAL (se verifica, no se pondera): respeto básico — sin acoso, sin mansplaining, sin conductas excluyentes. El umbral no entra en la ponderación: su incumplimiento verificado bloquea el nivel. Ver hoja «4. Ética del liderazgo».
-T6 ARTEFACTO · Estándares y playbooks; repositorio de evidencia; catálogo de intervenciones reutilizables; modelo de capacidades del Council.
-T9 COMPETENCIA · Stakeholder management; influencia; comunicación estratégica; facilitación; mentoring; priorización de portafolio.</t>
+          <t>META-CAPACIDAD: Criterio de escalamiento y liderazgo: decidir qué se estandariza, qué se deja variar y a qué ritmo se le puede exigir a un equipo, sosteniendo el equilibrio entre lo que el equipo produce y lo que el equipo puede sostener.
+OBJETIVO: Escalar conocimiento, prácticas y capacidades; desarrollar personas; sostener una cultura de decisión basada en evidencia.
+ENFOQUE: Evidencia acumulativa frente a estudio aislado; estandarizar frente a dejar variar; construir capacidad interna frente a resolver por encargo.
+METODOLOGÍA: ResearchOps, BehavioralOps y KnowledgeOps como sistemas de trabajo; gobernanza de estándares y de datos; capability building y modelos de desarrollo de personas; mejora continua.
+TÉCNICA: Conocimiento: repositorios y taxonomías de evidencia, activación y democratización del conocimiento, automatización de tareas operativas, trazabilidad. Liderazgo y equipo: feedback ascendente anónimo, observación estructurada de reuniones (habla, interrupciones y atribución de ideas), registro de asignación de oportunidades visibles, planes de desarrollo, entrevista de salida.
+MARCO: Systems thinking aplicado a la propia capacidad; modelo de madurez de la práctica; ciclo de mejora continua; el propio marco conductual aplicado al equipo — la conducta de quien lidera también es conducta observable.
+ARTEFACTO: Estándares y playbooks; repositorio de evidencia; catálogo de intervenciones reutilizables; modelo de capacidades del Council; tablero del equilibrio productividad–satisfacción del equipo.
+CALIDAD Y ÉTICA: Estándares metodológicos; gobernanza de datos, privacidad y trazabilidad; gestión de calidad. Ética del liderazgo, en dos partes que no se mezclan. EQUILIBRIO (se pondera): productividad del equipo ↔ satisfacción del equipo con la persona que lidera, leídas en el mismo periodo y nunca por separado. UMBRAL (se verifica, no se pondera): respeto básico, sin acoso, sin mansplaining, sin conductas excluyentes; su incumplimiento verificado bloquea el nivel y no entra en la ponderación.
+COMPETENCIAS: Stakeholder management; influencia; comunicación estratégica; facilitación; mentoring; priorización de portafolio.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Completar la columna Evidencias sugeridas
La columna venía vacía en el archivo original. Cuatro evidencias por
dimensión, cada una anclada a un artefacto real y no a una declaración
de la persona: el plan con sus alternativas descartadas, el problema
reencuadrado con su razonamiento, la intervención descartada por riesgo
ético, la lectura de un resultado negativo, el estándar adoptado sin
imposición.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tAd4V47q1GQgexet1HAzR
</commit_message>
<xml_diff>
--- a/matriz-expertiz/Propuesta_Matriz_expertiz_taxonomias.xlsx
+++ b/matriz-expertiz/Propuesta_Matriz_expertiz_taxonomias.xlsx
@@ -5062,7 +5062,14 @@
           <t>Define la estrategia de conocimiento e insights, conectando evidencia acumulativa para anticipar preguntas y orientar decisiones estratégicas.</t>
         </is>
       </c>
-      <c r="K6" s="8" t="n"/>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>· Un plan de investigación con la justificación del método frente a las alternativas descartadas.
+· Un estudio completo con su guía, criterio muestral y notas de campo.
+· Un set de insights trazables a la evidencia que los sustenta (verbatims, datos, fuentes).
+· Un caso en que la evidencia cambió la decisión que ya se iba a tomar.</t>
+        </is>
+      </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
           <t>Buscar: amplía y acelera la búsqueda de evidencia interna y externa.
@@ -5130,7 +5137,14 @@
           <t>Construye marcos estratégicos que transforman cómo la organización comprende problemas y oportunidades, influyendo en prioridades y decisiones de negocio</t>
         </is>
       </c>
-      <c r="K7" s="8" t="n"/>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>· Un problema reencuadrado: el enunciado inicial, el final y el razonamiento entre ambos.
+· Un mapa de oportunidades con los criterios de priorización explícitos.
+· Una decisión tomada con evidencia parcial, con el umbral de suficiencia declarado antes.
+· Una recomendación que se sostuvo ante negocio frente a objeciones.</t>
+        </is>
+      </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
           <t>Reencuadrar: propone diferentes formas de interpretar y formular un problema.
@@ -5198,7 +5212,14 @@
           <t>Define principios y modelos que transforman cómo RIMAC diseña decisiones, experiencias e intervenciones basadas en evidencia</t>
         </is>
       </c>
-      <c r="K8" s="8" t="n"/>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>· Una intervención conductual documentada: conducta objetivo, palanca elegida y por qué esa.
+· Principios y criterios de diseño que otro equipo usó después.
+· Un blueprint de orquestación a través de canales.
+· Una intervención descartada por desproporcionada o por riesgo ético, con el razonamiento escrito.</t>
+        </is>
+      </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
           <t>Idear: genera alternativas de conceptos, experiencias e intervenciones.
@@ -5266,7 +5287,14 @@
           <t>Define estándares y sistemas de experimentación y evidencia acumulativa que orientan decisiones estratégicas, escalamiento e inversión.</t>
         </is>
       </c>
-      <c r="K9" s="8" t="n"/>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>· Un diseño experimental completo: hipótesis, variables, regla de asignación y tamaño muestral.
+· Una lectura de resultados con tamaño de efecto y límites de validez declarados.
+· Dos decisiones resueltas con distinto nivel de rigor, con la justificación de cada una.
+· Un caso de resultado negativo en que se detuvo o se rehízo la intervención.</t>
+        </is>
+      </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
           <t>Formular: ayuda a convertir supuestos en hipótesis, variables y criterios de éxito.
@@ -5334,7 +5362,14 @@
           <t>Define la gobernanza y evolución de Customer Science, construyendo una capacidad organizacional ética, reconocida, acumulativa y escalable</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n"/>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>· Un estándar o playbook adoptado por otros sin imposición.
+· Evidencia reutilizada por alguien que no participó del estudio original.
+· El indicador de entrega del equipo y su feedback ascendente del mismo periodo, leídos juntos.
+· Un plan de desarrollo con progresión demostrable de otra persona.</t>
+        </is>
+      </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
           <t>Automatizar: reduce tareas operativas y repetitivas de ResearchOps y BehavioralOps.

</xml_diff>